<commit_message>
fix: add DSCR auto-calculation with detailed debt service breakdown
Added Section D2 with debt service items:
- Interest expenses
- Short-term repayments (bank, institutions, shareholders, commercial)
- Long-term repayments (bank, other, shareholders, bonds, leases)
- Total Debt Service (auto-sum)
- DSCR = EBITDA / Total Debt Service (auto-calculated)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/ebitda-dscr-calculation-2022-2024.xlsx
+++ b/public/templates/ebitda-dscr-calculation-2022-2024.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Financial Data'!$A$1:$F$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Financial Data'!$A$1:$F$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,12 +65,17 @@
       <sz val="10"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <i val="1"/>
       <color rgb="00999999"/>
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +118,12 @@
         <bgColor rgb="00EDF2F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFDE7"/>
+        <bgColor rgb="00FFFDE7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -140,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -174,9 +185,12 @@
     <xf numFmtId="10" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -544,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1276,110 +1290,389 @@
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="10" t="n">
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>D2. DSCR CALCULATION / PERHITUNGAN DSCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="21" t="inlineStr">
+        <is>
+          <t>Debt Servicing Items / Komponen Pembayaran Utang:</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr"/>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Interest Expenses / Beban Bunga</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Repayment of Short-term Liabilities / Pembayaran Utang Jangka Pendek:</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr"/>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bank Loans / Pinjaman Bank</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr"/>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Other Financial Institution Loans</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr"/>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Shareholder/Related Party Loans</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr"/>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Commercial Papers</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Repayment of Long-term Liabilities / Pembayaran Utang Jangka Panjang:</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr"/>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bank Loans / Pinjaman Bank</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr"/>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Other Source Loans</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr"/>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Shareholder Loans</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr"/>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Bonds Payable / Obligasi</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr"/>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Lease Liabilities / Sewa</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D53" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="n">
         <v>23</v>
       </c>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>DSCR (Debt Service Coverage Ratio)</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="inlineStr">
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>Total Debt Service / Total Pembayaran Utang</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D54" s="23">
+        <f>D42+D44+D45+D46+D47+D49+D50+D51+D52+D53</f>
+        <v/>
+      </c>
+      <c r="E54" s="23">
+        <f>E42+E44+E45+E46+E47+E49+E50+E51+E52+E53</f>
+        <v/>
+      </c>
+      <c r="F54" s="23">
+        <f>F42+F44+F45+F46+F47+F49+F50+F51+F52+F53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>DSCR (EBITDA / Total Debt Service)</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="D39" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
+      <c r="D55" s="20">
+        <f>IF(D54=0,0,D10/D54)</f>
+        <v/>
+      </c>
+      <c r="E55" s="20">
+        <f>IF(E54=0,0,E10/E54)</f>
+        <v/>
+      </c>
+      <c r="F55" s="20">
+        <f>IF(F54=0,0,F10/F54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
         <is>
           <t>E. CREDIT RATING / PERINGKAT KREDIT</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="21" t="inlineStr">
+    <row r="58">
+      <c r="B58" s="24" t="inlineStr">
         <is>
           <t>☐  DNDB</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D58" s="25" t="inlineStr">
         <is>
           <t>e.g. SA2</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="21" t="inlineStr">
+    <row r="59">
+      <c r="B59" s="24" t="inlineStr">
         <is>
           <t>☐  S&amp;P (Pefindo)</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D59" s="25" t="inlineStr">
         <is>
           <t>e.g. AA+</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="21" t="inlineStr">
+    <row r="60">
+      <c r="B60" s="24" t="inlineStr">
         <is>
           <t>☐  Moody's</t>
         </is>
       </c>
-      <c r="D44" s="22" t="inlineStr">
+      <c r="D60" s="25" t="inlineStr">
         <is>
           <t>e.g. Aaa</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="21" t="inlineStr">
+    <row r="61">
+      <c r="B61" s="24" t="inlineStr">
         <is>
           <t>☐  Fitch</t>
         </is>
       </c>
-      <c r="D45" s="22" t="inlineStr">
+      <c r="D61" s="25" t="inlineStr">
         <is>
           <t>e.g. AAA</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="21" t="inlineStr">
+    <row r="62">
+      <c r="B62" s="24" t="inlineStr">
         <is>
           <t>☐  Other</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="23" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="26" t="inlineStr">
         <is>
           <t>PT Bukit Asam (Persero) Tbk — PRIMA (Platform Registrasi, Informasi &amp; Manajemen Mitra)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A41:F41"/>
+  <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A40:F40"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A64:F64"/>
     <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A57:F57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>

<commit_message>
Update xlsx templates: currency dropdown and Total Liability rename
- C4 now has dropdown: "Thousand USD" / "Million IDR"
- All unit cells auto-update based on selected currency
- Renamed Total Debt to Total Liability

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/ebitda-dscr-calculation-2022-2024.xlsx
+++ b/public/templates/ebitda-dscr-calculation-2022-2024.xlsx
@@ -125,7 +125,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -147,11 +147,55 @@
         <color rgb="00D0D8E8"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D8E8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D8E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D8E8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D8E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D8E8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D8E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D8E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D8E8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -193,6 +237,8 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -586,7 +632,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Please fill in white boxes. Do not leave blank — fill with 0 if unknown. All data in USD.</t>
+          <t>Please fill in white boxes. Do not leave blank — fill with 0 if unknown.</t>
         </is>
       </c>
     </row>
@@ -598,7 +644,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Thousand USD</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -612,6 +658,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
@@ -644,6 +691,11 @@
           <t>A. INCOME STATEMENT / LAPORAN LABA RUGI</t>
         </is>
       </c>
+      <c r="B7" s="27" t="n"/>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="28" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n">
@@ -654,10 +706,9 @@
           <t>Revenue / Pendapatan</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C8" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D8" s="13" t="n">
         <v>0</v>
@@ -678,10 +729,9 @@
           <t>Gross Profit / Laba Kotor</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C9" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D9" s="13" t="n">
         <v>0</v>
@@ -702,10 +752,9 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C10" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D10" s="13" t="n">
         <v>0</v>
@@ -726,10 +775,9 @@
           <t>Net Income / Laba Bersih</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C11" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D11" s="13" t="n">
         <v>0</v>
@@ -750,10 +798,9 @@
           <t>Interest Expense / Beban Bunga</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C12" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D12" s="13" t="n">
         <v>0</v>
@@ -774,10 +821,9 @@
           <t>Taxes / Pajak</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C13" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D13" s="15" t="n">
         <v>0</v>
@@ -798,10 +844,9 @@
           <t>Depreciation / Depresiasi</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C14" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D14" s="15" t="n">
         <v>0</v>
@@ -822,10 +867,9 @@
           <t>Amortization / Amortisasi</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C15" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D15" s="15" t="n">
         <v>0</v>
@@ -887,12 +931,18 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
           <t>B. BALANCE SHEET / NERACA</t>
         </is>
       </c>
+      <c r="B19" s="27" t="n"/>
+      <c r="C19" s="27" t="n"/>
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="28" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n">
@@ -900,13 +950,12 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Total Debt / Total Utang</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+          <t>Total Liability / Total Liabilitas</t>
+        </is>
+      </c>
+      <c r="C20" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D20" s="13" t="n">
         <v>0</v>
@@ -927,10 +976,9 @@
           <t>Total Equity / Total Ekuitas</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C21" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D21" s="13" t="n">
         <v>0</v>
@@ -951,10 +999,9 @@
           <t>Total Assets / Total Aset (auto)</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C22" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D22" s="19">
         <f>D20+D21</f>
@@ -978,10 +1025,9 @@
           <t>Current Assets / Aset Lancar</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C23" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D23" s="13" t="n">
         <v>0</v>
@@ -1002,10 +1048,9 @@
           <t>Current Liabilities / Kewajiban Lancar</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C24" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D24" s="13" t="n">
         <v>0</v>
@@ -1026,10 +1071,9 @@
           <t>Interest Bearing Debt / Utang Berbunga</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C25" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D25" s="13" t="n">
         <v>0</v>
@@ -1048,10 +1092,9 @@
           <t>Net Worth / Kekayaan Bersih (auto)</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C26" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D26" s="19">
         <f>D22-D20</f>
@@ -1066,12 +1109,18 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
           <t>C. CASH FLOW / ARUS KAS</t>
         </is>
       </c>
+      <c r="B28" s="27" t="n"/>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="27" t="n"/>
+      <c r="E28" s="27" t="n"/>
+      <c r="F28" s="28" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n">
@@ -1082,10 +1131,9 @@
           <t>Operating Cash Flow / Arus Kas Operasi</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C29" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D29" s="13" t="n">
         <v>0</v>
@@ -1106,10 +1154,9 @@
           <t>Cash on Hand (Latest) / Kas Tersedia</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C30" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D30" s="13" t="n">
         <v>0</v>
@@ -1121,12 +1168,18 @@
         <v>0</v>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
           <t>D. FINANCIAL RATIOS / RASIO KEUANGAN (Auto-Calculated)</t>
         </is>
       </c>
+      <c r="B32" s="27" t="n"/>
+      <c r="C32" s="27" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="27" t="n"/>
+      <c r="F32" s="28" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="16" t="n">
@@ -1290,12 +1343,18 @@
         <v/>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
           <t>D2. DSCR CALCULATION / PERHITUNGAN DSCR</t>
         </is>
       </c>
+      <c r="B40" s="27" t="n"/>
+      <c r="C40" s="27" t="n"/>
+      <c r="D40" s="27" t="n"/>
+      <c r="E40" s="27" t="n"/>
+      <c r="F40" s="28" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="21" t="inlineStr">
@@ -1311,10 +1370,9 @@
           <t xml:space="preserve">  Interest Expenses / Beban Bunga</t>
         </is>
       </c>
-      <c r="C42" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C42" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D42" s="13" t="n">
         <v>0</v>
@@ -1340,10 +1398,9 @@
           <t xml:space="preserve">    Bank Loans / Pinjaman Bank</t>
         </is>
       </c>
-      <c r="C44" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C44" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D44" s="15" t="n">
         <v>0</v>
@@ -1362,10 +1419,9 @@
           <t xml:space="preserve">    Other Financial Institution Loans</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C45" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D45" s="15" t="n">
         <v>0</v>
@@ -1384,10 +1440,9 @@
           <t xml:space="preserve">    Shareholder/Related Party Loans</t>
         </is>
       </c>
-      <c r="C46" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C46" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D46" s="15" t="n">
         <v>0</v>
@@ -1406,10 +1461,9 @@
           <t xml:space="preserve">    Commercial Papers</t>
         </is>
       </c>
-      <c r="C47" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C47" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D47" s="15" t="n">
         <v>0</v>
@@ -1435,10 +1489,9 @@
           <t xml:space="preserve">    Bank Loans / Pinjaman Bank</t>
         </is>
       </c>
-      <c r="C49" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C49" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D49" s="15" t="n">
         <v>0</v>
@@ -1457,10 +1510,9 @@
           <t xml:space="preserve">    Other Source Loans</t>
         </is>
       </c>
-      <c r="C50" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C50" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D50" s="15" t="n">
         <v>0</v>
@@ -1479,10 +1531,9 @@
           <t xml:space="preserve">    Shareholder Loans</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C51" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D51" s="15" t="n">
         <v>0</v>
@@ -1501,10 +1552,9 @@
           <t xml:space="preserve">    Bonds Payable / Obligasi</t>
         </is>
       </c>
-      <c r="C52" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C52" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D52" s="15" t="n">
         <v>0</v>
@@ -1523,10 +1573,9 @@
           <t xml:space="preserve">    Lease Liabilities / Sewa</t>
         </is>
       </c>
-      <c r="C53" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C53" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D53" s="15" t="n">
         <v>0</v>
@@ -1547,10 +1596,9 @@
           <t>Total Debt Service / Total Pembayaran Utang</t>
         </is>
       </c>
-      <c r="C54" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
+      <c r="C54" s="12">
+        <f>IF($C$4="Thousand USD","Thousand USD","Million IDR")</f>
+        <v/>
       </c>
       <c r="D54" s="23">
         <f>D42+D44+D45+D46+D47+D49+D50+D51+D52+D53</f>
@@ -1592,12 +1640,18 @@
         <v/>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
           <t>E. CREDIT RATING / PERINGKAT KREDIT</t>
         </is>
       </c>
+      <c r="B57" s="27" t="n"/>
+      <c r="C57" s="27" t="n"/>
+      <c r="D57" s="27" t="n"/>
+      <c r="E57" s="27" t="n"/>
+      <c r="F57" s="28" t="n"/>
     </row>
     <row r="58">
       <c r="B58" s="24" t="inlineStr">
@@ -1654,6 +1708,7 @@
         </is>
       </c>
     </row>
+    <row r="63"/>
     <row r="64">
       <c r="A64" s="26" t="inlineStr">
         <is>
@@ -1674,6 +1729,11 @@
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="A57:F57"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Currency" error="Please select Thousand USD or Million IDR" promptTitle="Currency" prompt="Select currency unit" type="list">
+      <formula1>"Thousand USD,Million IDR"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>